<commit_message>
Them tai lieu ban giao 08_Ban_giao_Claude_Code.md
Ghi lai toan bo tinh trang thuc te + quyet dinh ky thuat cua phien
deploy vua roi (Supabase that, Cloudflare Workers thay vi Pages, bug
root directory da gap va cach fix, khac biet giua Tin tuc da lam va
spec blog.html goc). Dong bo lai CLAUDE.md/README.md/file Excel cho
khop trang thai thuc te (da lam that, khong con la ban nhap).
</commit_message>
<xml_diff>
--- a/01_Docs/Visa-Landing-Page_Tai_lieu.xlsx
+++ b/01_Docs/Visa-Landing-Page_Tai_lieu.xlsx
@@ -8931,7 +8931,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Dùng khi tiếp tục phát triển dự án bằng Claude Code | Xem đầy đủ tại CLAUDE.md ở thư mục gốc dự án | Cập nhật 2026-07-18</t>
+          <t>Dùng khi tiếp tục phát triển dự án bằng Claude Code | Xem đầy đủ tại CLAUDE.md ở thư mục gốc dự án | Cập nhật 2026-07-30</t>
         </is>
       </c>
     </row>
@@ -9026,12 +9026,12 @@
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>admin.html + supabase_setup.sql viết xong — CHƯA chạy (thiếu SUPABASE_URL/ANON_KEY)</t>
-        </is>
-      </c>
-      <c r="C9" s="14" t="inlineStr">
-        <is>
-          <t>☐ Chưa</t>
+          <t>admin.html + supabase_setup.sql — ĐÃ CHẠY THẬT, SUPABASE_URL/ANON_KEY đã điền (xem 08_Ban_giao_Claude_Code.md)</t>
+        </is>
+      </c>
+      <c r="C9" s="27" t="inlineStr">
+        <is>
+          <t>✓ Xong</t>
         </is>
       </c>
       <c r="D9" s="6" t="inlineStr"/>
@@ -9045,12 +9045,12 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Test case tại sheet 05_Kế hoạch — test trên Supabase Cloud thật</t>
+          <t>Đã test thủ công 1 phần (gửi lead thật, đăng nhập/đăng bài admin) — CHƯA chạy đủ 14 test case chính thức sheet 05_Kế hoạch</t>
         </is>
       </c>
       <c r="C10" s="14" t="inlineStr">
         <is>
-          <t>☐ Chưa</t>
+          <t>☐ Một phần</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr"/>
@@ -9064,12 +9064,12 @@
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>Chưa đưa lên Cloudflare Pages</t>
-        </is>
-      </c>
-      <c r="C11" s="14" t="inlineStr">
-        <is>
-          <t>☐ Chưa</t>
+          <t>Đã deploy thật qua Cloudflare Workers (không phải Pages) — https://topvisa.nguyennc1357.workers.dev</t>
+        </is>
+      </c>
+      <c r="C11" s="27" t="inlineStr">
+        <is>
+          <t>✓ Xong</t>
         </is>
       </c>
       <c r="D11" s="6" t="inlineStr"/>
@@ -9083,12 +9083,12 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Tài liệu spec đã có ở sheet 09 — CHƯA code</t>
+          <t>Đã làm bản rút gọn (section Tin tức trong index.html, không phải blog.html riêng như spec) — xem 08_Ban_giao_Claude_Code.md mục 6</t>
         </is>
       </c>
       <c r="C12" s="14" t="inlineStr">
         <is>
-          <t>☐ Chưa</t>
+          <t>☐ Một phần</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr"/>
@@ -9390,7 +9390,7 @@
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>(trống — cần điền theo 07_Huong_dan_Deploy.md Bước 1)</t>
+          <t>https://vvnjxvcdnzttcdufjjgo.supabase.co (đã điền thật)</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr"/>
@@ -9400,12 +9400,12 @@
     <row r="37" ht="16" customHeight="1">
       <c r="A37" s="6" t="inlineStr">
         <is>
-          <t>SUPABASE_ANON_KEY</t>
+          <t>SUPABASE_ANON_KEY (Publishable key)</t>
         </is>
       </c>
       <c r="B37" s="6" t="inlineStr">
         <is>
-          <t>(trống — cần điền)</t>
+          <t>sb_publishable_mp5Q5GRLV_ll8E4eNeivWw_aUv0q0xR (đã điền thật, an toàn public)</t>
         </is>
       </c>
       <c r="C37" s="6" t="inlineStr"/>

</xml_diff>